<commit_message>
Correct audit validation cells in model.xlsx
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/melkim/Documents/01 EDUCATION – SHIDLER DLeMBA/02-BUS 620-ECONOMICS /03 BUS 620 ECONOMICS ASSIGNMENTS /CASE 1 PERFECT COMPETITION /"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E5C5BCB5-A1D8-394A-A57E-574922B43596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{822154F7-083E-684D-8C1D-2F12352D3E12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="580" yWindow="1700" windowWidth="51200" windowHeight="28200" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4880" yWindow="600" windowWidth="46320" windowHeight="28200" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -111,7 +111,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="191">
   <si>
     <t>Perfect Competition — Model Inputs</t>
   </si>
@@ -650,9 +650,6 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>Tomatobed10:MP$551.89 vsLab $551</t>
-  </si>
-  <si>
     <t xml:space="preserve">The farm lab is displaying a whole dollar result but our model is more granular . It is uses the actual components to make the calculations that can be audited  </t>
   </si>
   <si>
@@ -684,6 +681,9 @@
   </si>
   <si>
     <t xml:space="preserve">The farm model results were based on calculations that can be audited and verified </t>
+  </si>
+  <si>
+    <t>Tomatobed10:MP$551.41 vs Lab $551</t>
   </si>
 </sst>
 </file>
@@ -815,7 +815,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -11263,7 +11263,7 @@
         <v>PASS</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>162</v>
@@ -11372,8 +11372,8 @@
       <c r="B11" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="C11" s="14">
-        <v>47776</v>
+      <c r="C11" s="14" t="s">
+        <v>159</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>178</v>
@@ -11399,8 +11399,8 @@
       <c r="B12" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="C12" s="14">
-        <v>47776</v>
+      <c r="C12" s="14" t="s">
+        <v>159</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>178</v>
@@ -11427,13 +11427,13 @@
         <v>172</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>178</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>173</v>
@@ -11463,7 +11463,7 @@
         <v>176</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>177</v>
@@ -11480,19 +11480,19 @@
     </row>
     <row r="15" spans="1:15" ht="64">
       <c r="A15" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="C15" s="10" t="s">
         <v>184</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>185</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>178</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
@@ -11507,19 +11507,19 @@
     </row>
     <row r="16" spans="1:15" ht="48">
       <c r="A16" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="10" t="s">
         <v>187</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>188</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>178</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>

</xml_diff>